<commit_message>
fix(services): update JSON report extraction and zero-default formatting for QO001, QI001, QC001, and MB001
</commit_message>
<xml_diff>
--- a/templates/QO001.xlsx
+++ b/templates/QO001.xlsx
@@ -1,17 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4506"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MahletTeklemariam\Documents\Monthly Report\2026\Monthly Report\NBE Repot\Sep 2026\Templ\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="11760"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="10245" windowHeight="6300"/>
   </bookViews>
   <sheets>
     <sheet name="CAP_ADQ_OFB_QO001" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725"/>
-  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <calcPr calcId="162913"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -19,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="35">
   <si>
     <t>CAP_ADQ_OFB_QO001</t>
   </si>
@@ -118,16 +123,22 @@
   </si>
   <si>
     <t>** Factor to be determined on a case- by- basis in consultation with the NBE.</t>
+  </si>
+  <si>
+    <t>0000001</t>
+  </si>
+  <si>
+    <t>2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -169,7 +180,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -200,8 +211,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="27">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -543,11 +560,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF00B050"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF00B050"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF00B050"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -637,64 +684,72 @@
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -756,7 +811,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -791,7 +846,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -968,16 +1023,16 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G39"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="47.5703125" customWidth="1"/>
     <col min="3" max="3" width="12.42578125" customWidth="1"/>
@@ -987,88 +1042,97 @@
     <col min="7" max="7" width="19.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="34" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36"/>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="37"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="39"/>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="37"/>
-      <c r="B6" s="38"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="39"/>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="40"/>
-      <c r="B7" s="41"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="41"/>
-      <c r="E7" s="42"/>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="34"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="35"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="37"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="35"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="37"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="38"/>
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="40"/>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>1</v>
       </c>
       <c r="B8" s="10"/>
-      <c r="C8" s="30"/>
+      <c r="C8" s="47" t="s">
+        <v>33</v>
+      </c>
       <c r="D8" s="2"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>2</v>
       </c>
       <c r="B9" s="11"/>
-      <c r="C9" s="30"/>
+      <c r="C9" s="48" t="s">
+        <v>34</v>
+      </c>
       <c r="D9" s="2"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="43" t="s">
+    <row r="10" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="43"/>
-      <c r="C10" s="31"/>
+      <c r="B10" s="41"/>
+      <c r="C10" s="49">
+        <v>46204</v>
+      </c>
       <c r="D10" s="2"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="43" t="s">
+    <row r="11" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="43"/>
-      <c r="C11" s="31"/>
+      <c r="B11" s="41"/>
+      <c r="C11" s="50">
+        <v>46295</v>
+      </c>
       <c r="D11" s="2"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="13" spans="1:7" ht="15.75" thickBot="1">
-      <c r="F13" s="44" t="s">
+    <row r="12" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F13" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="44"/>
-    </row>
-    <row r="14" spans="1:7" ht="32.25" thickTop="1">
-      <c r="A14" s="45" t="s">
+      <c r="G13" s="42"/>
+    </row>
+    <row r="14" spans="1:7" ht="32.25" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="47" t="s">
+      <c r="B14" s="45" t="s">
         <v>7</v>
       </c>
       <c r="C14" s="12" t="s">
@@ -1087,9 +1151,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="16.5" thickBot="1">
-      <c r="A15" s="46"/>
-      <c r="B15" s="48"/>
+    <row r="15" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="44"/>
+      <c r="B15" s="46"/>
       <c r="C15" s="4" t="s">
         <v>13</v>
       </c>
@@ -1106,7 +1170,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="15.75">
+    <row r="16" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="14">
         <v>10</v>
       </c>
@@ -1129,7 +1193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.75">
+    <row r="17" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="14">
         <v>11</v>
       </c>
@@ -1142,7 +1206,7 @@
       <c r="F17" s="7"/>
       <c r="G17" s="15"/>
     </row>
-    <row r="18" spans="1:7" ht="15.75">
+    <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="14">
         <v>11.1</v>
       </c>
@@ -1165,7 +1229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15.75">
+    <row r="19" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="14">
         <v>11.2</v>
       </c>
@@ -1188,7 +1252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15.75">
+    <row r="20" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="14">
         <v>11.3</v>
       </c>
@@ -1211,7 +1275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15.75">
+    <row r="21" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="14">
         <v>11.4</v>
       </c>
@@ -1234,7 +1298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15.75">
+    <row r="22" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="14">
         <v>12</v>
       </c>
@@ -1247,20 +1311,22 @@
       <c r="F22" s="7"/>
       <c r="G22" s="15"/>
     </row>
-    <row r="23" spans="1:7" ht="15.75">
+    <row r="23" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="14">
         <v>12.1</v>
       </c>
       <c r="B23" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="28"/>
+      <c r="C23" s="28">
+        <v>7065.2738391700004</v>
+      </c>
       <c r="D23" s="22">
         <v>0.5</v>
       </c>
       <c r="E23" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3532.6369195850002</v>
       </c>
       <c r="F23" s="7">
         <v>0</v>
@@ -1270,7 +1336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.75">
+    <row r="24" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="14">
         <v>12.2</v>
       </c>
@@ -1293,7 +1359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15.75">
+    <row r="25" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="14">
         <v>12.3</v>
       </c>
@@ -1316,30 +1382,32 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15.75">
+    <row r="26" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="14">
         <v>12.4</v>
       </c>
       <c r="B26" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="28"/>
+      <c r="C26" s="28">
+        <v>108526.8295061</v>
+      </c>
       <c r="D26" s="22">
         <v>0.5</v>
       </c>
       <c r="E26" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>54263.414753049998</v>
       </c>
       <c r="F26" s="7">
         <v>1</v>
       </c>
       <c r="G26" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="31.5">
+        <v>54263.414753049998</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A27" s="14">
         <v>13</v>
       </c>
@@ -1352,7 +1420,7 @@
       <c r="F27" s="7"/>
       <c r="G27" s="15"/>
     </row>
-    <row r="28" spans="1:7" ht="15.75">
+    <row r="28" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="14">
         <v>13.1</v>
       </c>
@@ -1375,7 +1443,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="15.75">
+    <row r="29" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="14">
         <v>13.2</v>
       </c>
@@ -1398,7 +1466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15.75">
+    <row r="30" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="14">
         <v>13.3</v>
       </c>
@@ -1421,30 +1489,32 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15.75">
+    <row r="31" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="14">
         <v>13.4</v>
       </c>
       <c r="B31" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="28"/>
+      <c r="C31" s="28">
+        <v>2976.8396095399999</v>
+      </c>
       <c r="D31" s="22">
         <v>0.5</v>
       </c>
       <c r="E31" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1488.4198047699999</v>
       </c>
       <c r="F31" s="7">
         <v>1</v>
       </c>
       <c r="G31" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="15.75">
+        <v>1488.4198047699999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="14">
         <v>14</v>
       </c>
@@ -1457,7 +1527,7 @@
       <c r="F32" s="7"/>
       <c r="G32" s="15"/>
     </row>
-    <row r="33" spans="1:7" ht="15.75">
+    <row r="33" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="14">
         <v>14.1</v>
       </c>
@@ -1480,7 +1550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15.75">
+    <row r="34" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="14">
         <v>14.2</v>
       </c>
@@ -1503,14 +1573,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15.75">
+    <row r="35" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="14">
         <v>14.3</v>
       </c>
       <c r="B35" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C35" s="28"/>
+      <c r="C35" s="28">
+        <v>0</v>
+      </c>
       <c r="D35" s="22">
         <v>0.2</v>
       </c>
@@ -1526,30 +1598,32 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15.75">
+    <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="14">
         <v>14.4</v>
       </c>
       <c r="B36" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="C36" s="28"/>
+      <c r="C36" s="28">
+        <v>153830.89494134998</v>
+      </c>
       <c r="D36" s="22">
         <v>0.2</v>
       </c>
       <c r="E36" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>30766.178988269996</v>
       </c>
       <c r="F36" s="7">
         <v>1</v>
       </c>
       <c r="G36" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="16.5" thickBot="1">
+        <v>30766.178988269996</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="14">
         <v>15</v>
       </c>
@@ -1562,7 +1636,7 @@
       <c r="F37" s="7"/>
       <c r="G37" s="16"/>
     </row>
-    <row r="38" spans="1:7" ht="16.5" thickBot="1">
+    <row r="38" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="17">
         <v>16</v>
       </c>
@@ -1575,19 +1649,19 @@
       <c r="F38" s="20"/>
       <c r="G38" s="24">
         <f>SUM(G16:G37)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="31.5" customHeight="1" thickTop="1">
-      <c r="A39" s="32" t="s">
+        <v>86518.013546089991</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="31.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="B39" s="33"/>
-      <c r="C39" s="33"/>
-      <c r="D39" s="33"/>
-      <c r="E39" s="33"/>
-      <c r="F39" s="33"/>
-      <c r="G39" s="33"/>
+      <c r="B39" s="31"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="31"/>
+      <c r="E39" s="31"/>
+      <c r="F39" s="31"/>
+      <c r="G39" s="31"/>
     </row>
   </sheetData>
   <sheetProtection password="CF68" sheet="1" objects="1" scenarios="1"/>

</xml_diff>